<commit_message>
Literature review of 13 relevant papers
</commit_message>
<xml_diff>
--- a/docs/Papers/Literature Review.xlsx
+++ b/docs/Papers/Literature Review.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Thompson Rivers University\3rd Semester\Grad Project on Data Science\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1E95B2E-FD05-4A9F-B5E0-D1B047A6D562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A50C48-E473-4801-8857-8CC553E50E4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F4EAAAAA-136C-4ECC-B9E1-E975647880FD}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F4EAAAAA-136C-4ECC-B9E1-E975647880FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Literature Review" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
   <si>
     <t>No.</t>
   </si>
@@ -303,6 +303,78 @@
   </si>
   <si>
     <t>Extend framework to multi-domain, multilingual retention engines with continuous learning and cloud deployment.</t>
+  </si>
+  <si>
+    <t>Valentini et al. (2025)</t>
+  </si>
+  <si>
+    <t>Leveraging LLM-Powered Multi-Agent Systems to Enhance Customer Experience</t>
+  </si>
+  <si>
+    <t>Thakkar &amp; Yadav (2024)</t>
+  </si>
+  <si>
+    <t>Personalized Recommendation Systems Using Multimodal, Autonomous, Multi-Agent Systems</t>
+  </si>
+  <si>
+    <t>Sandhya et al. (2019)</t>
+  </si>
+  <si>
+    <t>Feature Intersection for Agent-Based Customer Churn Prediction</t>
+  </si>
+  <si>
+    <t>LLM-based multi-agent system (SofAgent), GPT-4o agents, knowledge-grounded retrieval over external KBs</t>
+  </si>
+  <si>
+    <t>Coordination overhead; occasional failure on nuanced constraints (FMR); relies on curated KB freshness.</t>
+  </si>
+  <si>
+    <t>API rate limits; hardware/compute constraints; limited large-scale A/B validation.</t>
+  </si>
+  <si>
+    <t>Rules static; telecom-only; limited micro-behavior evolution and cross-domain tests.</t>
+  </si>
+  <si>
+    <t>Reduced hallucination from 88.3% → 3.3%; improved factual accuracy = 74.17% on 120 complex retail queries via manager–specialist agent orchestration and KB grounding.</t>
+  </si>
+  <si>
+    <t>Provides architectural basis for a multi-agent decision layer in your engine (Manager + specialized agents for churn, recs, optimization).</t>
+  </si>
+  <si>
+    <t>First knowledge-grounded multi-agent LLM pipeline showing large reliability gains over single-agent LLMs in CX settings.</t>
+  </si>
+  <si>
+    <t>Add multimodal inputs (image/text), richer orchestration policies, and auto-KB refresh for evolving catalogs and policies.</t>
+  </si>
+  <si>
+    <t>Gemini-1.5 Pro, LLaMA-70B; Multimodal (text+image) agents; Groq LPU inference; LangChain/CrewAI orchestration</t>
+  </si>
+  <si>
+    <t>Achieved NDCG ≈ 0.83, Recall ≈ 0.6, F1 ≈ 0.6; multimodal agent adds visual discovery; Groq LPU cut latency from minutes → milliseconds for interactive UX.</t>
+  </si>
+  <si>
+    <t>Reinforces multimodal perception and autonomous agent collaboration for real-time personalization in your intervention loop.</t>
+  </si>
+  <si>
+    <t>Combines visual similarity search with LLM agents and low-latency inference, improving UX and conversion paths.</t>
+  </si>
+  <si>
+    <t>Scale via distributed inference, add online learning from clicks, and extend to multi-channel (app/web/email) personalization.</t>
+  </si>
+  <si>
+    <t>Intersection-Randomized Algorithm (IRA) + MapReduce for de-dup; Agent-Based Modeling; affinity propagation</t>
+  </si>
+  <si>
+    <t>On 18-month telecom logs: 95.8% churn accuracy; ~50% runtime reduction (e.g., 90s→50s for 50k users) by removing redundancy; agents simulate churn/retention states (CH_A/R_A/nCoR).</t>
+  </si>
+  <si>
+    <t>Provides agent-based simulation blueprint and big-data pre-processing (IRA) for scalable churn pipelines.</t>
+  </si>
+  <si>
+    <t>Hybrid Big Data + ABM framework; novel IRA pre-processing to cut cost while preserving predictive signal.</t>
+  </si>
+  <si>
+    <t>Add ML-learned agent rules, temporal behavior evolution, and validate on e-commerce/banking with streaming/real-time features.</t>
   </si>
 </sst>
 </file>
@@ -745,7 +817,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63EDF593-A152-4E52-8904-295059C2C56B}">
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.33203125" customWidth="1"/>
@@ -759,7 +831,7 @@
     <col min="9" max="9" width="54.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -788,7 +860,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -817,7 +889,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -846,7 +918,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -875,7 +947,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>4</v>
       </c>
@@ -904,7 +976,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>5</v>
       </c>
@@ -933,7 +1005,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
         <v>6</v>
       </c>
@@ -962,7 +1034,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>7</v>
       </c>
@@ -991,7 +1063,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A9" s="8">
         <v>8</v>
       </c>
@@ -1020,7 +1092,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>9</v>
       </c>
@@ -1049,7 +1121,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A11" s="8">
         <v>10</v>
       </c>
@@ -1078,16 +1150,127 @@
         <v>88</v>
       </c>
     </row>
+    <row r="12" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="8">
+        <v>11</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="8">
+        <v>12</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="I13" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="J13" s="2"/>
+    </row>
+    <row r="14" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="8">
+        <v>13</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="18" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+    </row>
+    <row r="19" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+    </row>
     <row r="20" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
     </row>
     <row r="21" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C21" s="3"/>
@@ -1177,28 +1360,6 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
     </row>
-    <row r="29" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-    </row>
-    <row r="30" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Literature review of 16 relevant papers
</commit_message>
<xml_diff>
--- a/docs/Papers/Literature Review.xlsx
+++ b/docs/Papers/Literature Review.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Thompson Rivers University\3rd Semester\Grad Project on Data Science\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Thompson Rivers University\3rd Semester\Grad Project on Data Science\Final Year Design Project\hyper-personalized-customer-engine\docs\Papers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A50C48-E473-4801-8857-8CC553E50E4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB7FFDB-995E-483D-ACFF-A085F9BF9F04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F4EAAAAA-136C-4ECC-B9E1-E975647880FD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="137">
   <si>
     <t>No.</t>
   </si>
@@ -375,13 +375,205 @@
   </si>
   <si>
     <t>Add ML-learned agent rules, temporal behavior evolution, and validate on e-commerce/banking with streaming/real-time features.</t>
+  </si>
+  <si>
+    <t>Cenggoro et al. (2021)</t>
+  </si>
+  <si>
+    <t>Deep Learning as a Vector Embedding Model for Customer Churn</t>
+  </si>
+  <si>
+    <t>Limited to small-scale telecom dataset; model lacks temporal awareness and real-time retraining; explainability limited to 2-D visualization.</t>
+  </si>
+  <si>
+    <t>Deep Neural Network with categorical embedding layers, weighted Softmax loss, t-SNE visualization, and cluster-based similarity metrics</t>
+  </si>
+  <si>
+    <t>Developed an explainable churn model using vector embedding for 3,333 telecom customers. The weighted Softmax loss (3:7) improved F1 Score to 81.16%, outperforming unweighted models. t-SNE visualizations revealed two churn clusters: one convertible (potentially recoverable) and one irrecoverable.</t>
+  </si>
+  <si>
+    <t>Introduces a representation-learning foundation for your project’s customer embedding and churn-vector space module, supporting interpretable segmentation and intervention targeting.</t>
+  </si>
+  <si>
+    <t>Pioneered the use of vector embeddings as interpretable representations for churn behavior. Demonstrated that embedded feature vectors can separate loyal vs. churning users and identify sub-clusters for retention targeting.</t>
+  </si>
+  <si>
+    <t>Extend to temporal vector embeddings, integrate cosine-distance or triplet-loss training, and deploy online-learning churn embeddings within multi-agent decision pipelines.</t>
+  </si>
+  <si>
+    <t>Saha et al. (2024)</t>
+  </si>
+  <si>
+    <t>ChurnNet: Deep Learning Enhanced Customer Churn Prediction in the Telecommunication Industry</t>
+  </si>
+  <si>
+    <t>High model complexity; no interpretability integration; centralized training only; requires large computational resources.</t>
+  </si>
+  <si>
+    <t>Vu (2024)</t>
+  </si>
+  <si>
+    <t>Predict Customer Churn Using Combination Deep Learning Networks Model</t>
+  </si>
+  <si>
+    <t>Domain-limited to banking data; deep layers remain black-box; static data snapshot; high compute cost for multi-model training.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Hybrid </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1D CNN with Residual Blocks, Squeeze-and-Excitation (SE), and Spatial Attention Modules (SAM); evaluated with SMOTE, SMOTE-Tomek, SMOTE-ENN balancing</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Outperformed 9 baselines (Logistic, RF, SVM, CNN, LSTM, GRU); achieved up to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>97.52% accuracy, F1 &gt; 96%, and AUC improvement of 4–6%; combined residual + attention mechanisms for robust feature learning.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Informs </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Deep Feature Learning (Phase 2) and Predictive Intelligence Layer (Phase 3) through attention-based modeling of customer attributes and churn-driving signals.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Introduced </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Residual-SE-SAM fusion for channel–spatial attention in tabular churn data; advanced feature extraction beyond conventional deep models.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Extend via </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>federated learning, Explainable AI (SHAP/LIME) integration, and data augmentation for streaming churn prediction.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Stacked Ensemble:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Three DNNs (ReLU/Tanh + RMSProp/Adam) as base models + Logistic Regression meta-classifier; optimized over 220 epochs</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Reached </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Accuracy = 96.60%, F1 = 91.07%, surpassing XGBoost, RNN, and LSTM by 4–7%; meta-layer improved interpretability and stability; balanced performance and transparency.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Supports </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hybrid Deep Learning Framework (Phase 3) — shows how ensemble-level fusion enhances predictive accuracy and interpretability in churn modeling.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Proposed a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>two-tier hybrid model combining deep learning with logistic regression; proved that ensemble diversity improves robustness and generalization.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Integrate </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Explainable AI (SHAP/LIME) for transparency; extend to temporal deep models (LSTM/Transformer); deploy cloud-scalable pipelines for real-time churn prediction.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -417,6 +609,13 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -454,7 +653,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -472,13 +671,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -820,15 +1013,15 @@
   <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.33203125" customWidth="1"/>
-    <col min="2" max="2" width="34.88671875" customWidth="1"/>
-    <col min="3" max="3" width="108.5546875" customWidth="1"/>
-    <col min="4" max="4" width="120.77734375" customWidth="1"/>
-    <col min="5" max="5" width="94.88671875" style="5" customWidth="1"/>
-    <col min="6" max="6" width="87.109375" style="5" customWidth="1"/>
-    <col min="7" max="7" width="53.44140625" customWidth="1"/>
+    <col min="1" max="1" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="106.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="119.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="94.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="86.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="69.33203125" customWidth="1"/>
     <col min="8" max="8" width="56.109375" customWidth="1"/>
-    <col min="9" max="9" width="54.77734375" customWidth="1"/>
+    <col min="9" max="9" width="69.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
@@ -844,402 +1037,490 @@
       <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="6" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="8">
+      <c r="A2" s="7">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="7" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="8">
+      <c r="A3" s="7">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="7" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="8">
+      <c r="A4" s="7">
         <v>3</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="7" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="8">
+      <c r="A5" s="7">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I5" s="7" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="8">
+      <c r="A6" s="7">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="I6" s="7" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="8">
+      <c r="A7" s="7">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="7" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="8">
+    <row r="8" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="7">
         <v>7</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="I8" s="9" t="s">
+      <c r="I8" s="7" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="8">
+    <row r="9" spans="1:10" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="7">
         <v>8</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="I9" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8">
+    <row r="10" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="7">
         <v>9</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="I10" s="9" t="s">
+      <c r="I10" s="7" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="8">
+      <c r="A11" s="7">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="7" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="8">
+    <row r="12" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="7">
         <v>11</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="H12" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="I12" s="7" t="s">
         <v>102</v>
       </c>
       <c r="J12" s="2"/>
     </row>
-    <row r="13" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="8">
+    <row r="13" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="7">
         <v>12</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="H13" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="I13" s="9" t="s">
+      <c r="I13" s="7" t="s">
         <v>107</v>
       </c>
       <c r="J13" s="2"/>
     </row>
     <row r="14" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="8">
+      <c r="A14" s="7">
         <v>13</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="H14" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="I14" s="9" t="s">
+      <c r="I14" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="18" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="7">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="7">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="J16" s="2"/>
+    </row>
+    <row r="17" spans="1:11" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="7">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
@@ -1250,7 +1531,7 @@
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
     </row>
-    <row r="19" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="4"/>
@@ -1261,7 +1542,7 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
     </row>
-    <row r="20" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="4"/>
@@ -1272,7 +1553,7 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
     </row>
-    <row r="21" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="4"/>
@@ -1283,7 +1564,7 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="4"/>
@@ -1294,7 +1575,7 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="4"/>
@@ -1305,7 +1586,7 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="4"/>
@@ -1316,7 +1597,7 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="4"/>
@@ -1327,7 +1608,7 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="4"/>
@@ -1338,7 +1619,7 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="4"/>
@@ -1349,7 +1630,7 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
     </row>
-    <row r="28" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="4"/>

</xml_diff>